<commit_message>
TAREFAS DE Funções Financeiras PARCIALMENTE CONCLUÍDAS
</commit_message>
<xml_diff>
--- a/Avancado/15 - Controle de Formulários.xlsx
+++ b/Avancado/15 - Controle de Formulários.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9577CA-3A61-4559-9516-2A2ED14ACDBB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Aplicação" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,8 +24,12 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -29,15 +39,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -45,12 +61,101 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -66,6 +171,69 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>946897</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>112059</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1821589" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CaixaDeTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE048A0B-F6BC-4ABF-99C9-0D102C6DA1DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1137397" y="112059"/>
+          <a:ext cx="1821589" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:t>Aplicações Financeiras</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +498,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="2" max="3" width="27.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TAREFA 15 parcialmente concluída
</commit_message>
<xml_diff>
--- a/Avancado/15 - Controle de Formulários.xlsx
+++ b/Avancado/15 - Controle de Formulários.xlsx
@@ -2,20 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
-  <workbookPr/>
+  <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9577CA-3A61-4559-9516-2A2ED14ACDBB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED31E21-0E14-4562-9D2D-FDF169719729}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aplicação" sheetId="1" r:id="rId1"/>
+    <sheet name="Cadastro" sheetId="2" r:id="rId2"/>
+    <sheet name="Dados" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,18 +27,98 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>Pagamento Mensal</t>
+  </si>
+  <si>
+    <t>Taxa Mensal</t>
+  </si>
+  <si>
+    <t>Período</t>
+  </si>
+  <si>
+    <t>Valor Futuro</t>
+  </si>
+  <si>
+    <t>Valor de Rendimento</t>
+  </si>
+  <si>
+    <t>Nome:</t>
+  </si>
+  <si>
+    <t>Idade:</t>
+  </si>
+  <si>
+    <t>Gênero:</t>
+  </si>
+  <si>
+    <t>Profissão</t>
+  </si>
+  <si>
+    <t>Renda:</t>
+  </si>
+  <si>
+    <t>Profissão:</t>
+  </si>
+  <si>
+    <t>Luiz Henrique Vidal Araujo</t>
+  </si>
+  <si>
+    <t>Técnico</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Idade</t>
+  </si>
+  <si>
+    <t>Gênero</t>
+  </si>
+  <si>
+    <t>Renda</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -53,7 +135,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -141,11 +223,123 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -156,9 +350,48 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -173,16 +406,44 @@
 </styleSheet>
 </file>
 
+<file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="22" fmlaLink="$C$2" horiz="1" inc="100" max="30000" min="100" page="1000" val="1100"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="22" fmlaLink="$D$4" max="120" min="1" page="10" val="12"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp3.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="22" fmlaLink="$C$6" horiz="1" max="360" min="1" page="10" val="7"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="GBox" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp5.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Radio" checked="Checked" firstButton="1" fmlaLink="$F$6" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp6.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Radio" lockText="1" noThreeD="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp7.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="22" fmlaLink="$H$2" max="30000" page="10" val="0"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>946897</xdr:colOff>
+      <xdr:colOff>960504</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>112059</xdr:rowOff>
+      <xdr:rowOff>20211</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1821589" cy="311496"/>
+    <xdr:ext cx="2335191" cy="374141"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="CaixaDeTexto 1">
@@ -196,13 +457,16 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1137397" y="112059"/>
-          <a:ext cx="1821589" cy="311496"/>
+          <a:off x="1151004" y="20211"/>
+          <a:ext cx="2335191" cy="374141"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
@@ -221,11 +485,34 @@
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
           <a:spAutoFit/>
+          <a:scene3d>
+            <a:camera prst="orthographicFront"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="18600000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d extrusionH="450850">
+            <a:bevelT w="38100" h="38100"/>
+            <a:bevelB w="38100" h="38100"/>
+          </a:sp3d>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:rPr lang="pt-BR" sz="1800" b="1">
+              <a:ln w="6350" cap="flat">
+                <a:noFill/>
+                <a:bevel/>
+              </a:ln>
+              <a:pattFill prst="dkUpDiag">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+            </a:rPr>
             <a:t>Aplicações Financeiras</a:t>
           </a:r>
         </a:p>
@@ -233,6 +520,559 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>5998</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>16933</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1823862</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>178858</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1025" name="Scroll Bar 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1025"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF3CCE43-6AC5-42BA-BB27-997071B5A52A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>14464</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>203553</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>141110</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>208137</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1026" name="Spinner 2" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1026"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7287C11-02A2-4288-B0D6-4250D2A4BF02}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>10583</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>21520</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1820333</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>183445</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1028" name="Scroll Bar 4" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1028"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09F984CA-D1D4-4FDA-8771-DBEFB250ED26}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>95249</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>149087</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>447260</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>103533</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2049" name="Group Box 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2049"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D433A27E-2AE1-4C5E-8F26-F9402313511C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:noFill/>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="none" lIns="45720" tIns="54864" rIns="0" bIns="0" anchor="t" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Segoe UI"/>
+                  <a:cs typeface="Segoe UI"/>
+                </a:rPr>
+                <a:t>Sexo</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>174763</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>79512</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>583924</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>79512</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2054" name="Option Button 6" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2054"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2AA35B03-050D-4D35-AA53-708A452342C7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="45720" tIns="54864" rIns="0" bIns="54864" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Segoe UI"/>
+                  <a:cs typeface="Segoe UI"/>
+                </a:rPr>
+                <a:t>M</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>12424</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>78685</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>381000</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>78685</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2055" name="Option Button 7" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2055"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{540A49F1-4367-496D-8478-34087AC2F672}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="45720" tIns="54864" rIns="0" bIns="54864" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="pt-BR" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Segoe UI"/>
+                  <a:cs typeface="Segoe UI"/>
+                </a:rPr>
+                <a:t>F</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>115956</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>128380</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>443119</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>41412</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="[0]!Enviar" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="Retângulo: Cantos Arredondados 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29A957F4-C0BA-476D-90BC-3322C4E32FF1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3801717" y="1395619"/>
+          <a:ext cx="935935" cy="335445"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst>
+            <a:gd name="adj" fmla="val 19149"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg2">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="44450" dist="27940" dir="5400000" algn="ctr">
+            <a:srgbClr val="000000">
+              <a:alpha val="32000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+        <a:scene3d>
+          <a:camera prst="orthographicFront">
+            <a:rot lat="0" lon="0" rev="0"/>
+          </a:camera>
+          <a:lightRig rig="balanced" dir="t">
+            <a:rot lat="0" lon="0" rev="8700000"/>
+          </a:lightRig>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT w="190500" h="38100" prst="coolSlant"/>
+        </a:sp3d>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100"/>
+            <a:t>Enviar</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>66675</xdr:colOff>
+          <xdr:row>0</xdr:row>
+          <xdr:rowOff>85725</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>304800</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>104775</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3073" name="Spinner 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s3073"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD646070-E557-4DD9-BF06-C42FF75D1D5E}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -498,7 +1338,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Planilha1"/>
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -506,67 +1347,92 @@
     <col min="2" max="3" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="B2" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="12">
+        <v>1100</v>
+      </c>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13">
+        <f>D4/100</f>
+        <v>0.12</v>
+      </c>
+      <c r="D4" s="14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="B6" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="11">
+        <v>7</v>
+      </c>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
+      <c r="B8" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="15">
+        <f>FV(C4,C6,-C2,0,0)</f>
+        <v>11097.912901222409</v>
+      </c>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="16">
+        <f>C8-(C2*C6)</f>
+        <v>3397.9129012224093</v>
+      </c>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -574,6 +1440,368 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1025" r:id="rId4" name="Scroll Bar 1">
+              <controlPr defaultSize="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>9525</xdr:colOff>
+                    <xdr:row>2</xdr:row>
+                    <xdr:rowOff>19050</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1819275</xdr:colOff>
+                    <xdr:row>2</xdr:row>
+                    <xdr:rowOff>180975</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1026" r:id="rId5" name="Spinner 2">
+              <controlPr defaultSize="0" autoPict="0">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>3</xdr:col>
+                    <xdr:colOff>19050</xdr:colOff>
+                    <xdr:row>2</xdr:row>
+                    <xdr:rowOff>200025</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>3</xdr:col>
+                    <xdr:colOff>142875</xdr:colOff>
+                    <xdr:row>3</xdr:row>
+                    <xdr:rowOff>209550</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1028" r:id="rId6" name="Scroll Bar 4">
+              <controlPr defaultSize="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>9525</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>19050</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1819275</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>180975</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE70762-C831-41CC-A23A-E19CECDB04CC}">
+  <sheetPr codeName="Planilha2"/>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="20"/>
+    </row>
+    <row r="2" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="21"/>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="22"/>
+    </row>
+    <row r="3" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="21"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="22"/>
+    </row>
+    <row r="4" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21"/>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="22"/>
+    </row>
+    <row r="5" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="21"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="22"/>
+    </row>
+    <row r="6" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="11" t="str">
+        <f>IF(C2="","",IF(F6=1,"Masculino","Feminino"))</f>
+        <v>Masculino</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="22"/>
+    </row>
+    <row r="8" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="22"/>
+    </row>
+    <row r="9" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="22"/>
+    </row>
+    <row r="10" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="21"/>
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="12">
+        <v>2000</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="21"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="22"/>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="23"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="25"/>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="2049" r:id="rId3" name="Group Box 1">
+              <controlPr defaultSize="0" autoFill="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>3</xdr:col>
+                    <xdr:colOff>95250</xdr:colOff>
+                    <xdr:row>4</xdr:row>
+                    <xdr:rowOff>152400</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>4</xdr:col>
+                    <xdr:colOff>447675</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>104775</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="2054" r:id="rId4" name="Option Button 6">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>3</xdr:col>
+                    <xdr:colOff>171450</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>76200</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>3</xdr:col>
+                    <xdr:colOff>581025</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>76200</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="2055" r:id="rId5" name="Option Button 7">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>4</xdr:col>
+                    <xdr:colOff>9525</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>76200</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>4</xdr:col>
+                    <xdr:colOff>381000</xdr:colOff>
+                    <xdr:row>6</xdr:row>
+                    <xdr:rowOff>76200</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43C7F98-EBD0-473E-BF7A-17630AB92799}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="18.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
+    <col min="5" max="6" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" customWidth="1"/>
+    <col min="8" max="8" width="2.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="28"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="H2" s="28">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="3073" r:id="rId3" name="Spinner 1">
+              <controlPr defaultSize="0" autoPict="0">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>6</xdr:col>
+                    <xdr:colOff>66675</xdr:colOff>
+                    <xdr:row>0</xdr:row>
+                    <xdr:rowOff>85725</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>6</xdr:col>
+                    <xdr:colOff>304800</xdr:colOff>
+                    <xdr:row>2</xdr:row>
+                    <xdr:rowOff>104775</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
 </worksheet>
 </file>
</xml_diff>